<commit_message>
Replace Gemini API classifier with rule-based keyword classifier
Eliminates dependency on Gemini API free tier (quota too low for monthly use).
Rule-based matching covers 23 categories with Japanese/English keyword lists.
No API calls required — instant classification, no rate limits.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/MarketNews-202604.xlsx
+++ b/output/MarketNews-202604.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y109"/>
+  <dimension ref="A1:Y91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -819,7 +819,9 @@
         </is>
       </c>
       <c r="C3" s="11" t="n"/>
-      <c r="D3" s="11" t="n"/>
+      <c r="D3" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E3" s="11" t="n"/>
       <c r="F3" s="11" t="n"/>
       <c r="G3" s="11" t="n"/>
@@ -856,13 +858,17 @@
         </is>
       </c>
       <c r="C4" s="15" t="n"/>
-      <c r="D4" s="15" t="n"/>
+      <c r="D4" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E4" s="15" t="n"/>
       <c r="F4" s="15" t="n"/>
       <c r="G4" s="15" t="n"/>
       <c r="H4" s="15" t="n"/>
       <c r="I4" s="15" t="n"/>
-      <c r="J4" s="15" t="n"/>
+      <c r="J4" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K4" s="15" t="n"/>
       <c r="L4" s="15" t="n"/>
       <c r="M4" s="15" t="n"/>
@@ -877,9 +883,7 @@
       <c r="V4" s="15" t="n"/>
       <c r="W4" s="15" t="n"/>
       <c r="X4" s="15" t="n"/>
-      <c r="Y4" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -893,13 +897,17 @@
         </is>
       </c>
       <c r="C5" s="11" t="n"/>
-      <c r="D5" s="11" t="n"/>
+      <c r="D5" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E5" s="11" t="n"/>
       <c r="F5" s="11" t="n"/>
       <c r="G5" s="11" t="n"/>
       <c r="H5" s="11" t="n"/>
       <c r="I5" s="11" t="n"/>
-      <c r="J5" s="11" t="n"/>
+      <c r="J5" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="K5" s="11" t="n"/>
       <c r="L5" s="11" t="n"/>
       <c r="M5" s="11" t="n"/>
@@ -913,10 +921,10 @@
       <c r="U5" s="11" t="n"/>
       <c r="V5" s="11" t="n"/>
       <c r="W5" s="11" t="n"/>
-      <c r="X5" s="11" t="n"/>
-      <c r="Y5" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="X5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="11" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -930,7 +938,9 @@
         </is>
       </c>
       <c r="C6" s="15" t="n"/>
-      <c r="D6" s="15" t="n"/>
+      <c r="D6" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="15" t="n"/>
       <c r="G6" s="15" t="n"/>
@@ -945,15 +955,15 @@
       <c r="P6" s="15" t="n"/>
       <c r="Q6" s="15" t="n"/>
       <c r="R6" s="15" t="n"/>
-      <c r="S6" s="15" t="n"/>
+      <c r="S6" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T6" s="15" t="n"/>
       <c r="U6" s="15" t="n"/>
       <c r="V6" s="15" t="n"/>
       <c r="W6" s="15" t="n"/>
       <c r="X6" s="15" t="n"/>
-      <c r="Y6" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y6" s="15" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -967,7 +977,9 @@
         </is>
       </c>
       <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
+      <c r="D7" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E7" s="11" t="n"/>
       <c r="F7" s="11" t="n"/>
       <c r="G7" s="11" t="n"/>
@@ -982,15 +994,17 @@
       <c r="P7" s="11" t="n"/>
       <c r="Q7" s="11" t="n"/>
       <c r="R7" s="11" t="n"/>
-      <c r="S7" s="11" t="n"/>
+      <c r="S7" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T7" s="11" t="n"/>
       <c r="U7" s="11" t="n"/>
       <c r="V7" s="11" t="n"/>
       <c r="W7" s="11" t="n"/>
-      <c r="X7" s="11" t="n"/>
-      <c r="Y7" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="X7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -1004,7 +1018,9 @@
         </is>
       </c>
       <c r="C8" s="15" t="n"/>
-      <c r="D8" s="15" t="n"/>
+      <c r="D8" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E8" s="15" t="n"/>
       <c r="F8" s="15" t="n"/>
       <c r="G8" s="15" t="n"/>
@@ -1024,10 +1040,10 @@
       <c r="U8" s="15" t="n"/>
       <c r="V8" s="15" t="n"/>
       <c r="W8" s="15" t="n"/>
-      <c r="X8" s="15" t="n"/>
-      <c r="Y8" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="X8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1041,7 +1057,9 @@
         </is>
       </c>
       <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
+      <c r="D9" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E9" s="11" t="n"/>
       <c r="F9" s="11" t="n"/>
       <c r="G9" s="11" t="n"/>
@@ -1078,13 +1096,17 @@
         </is>
       </c>
       <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
+      <c r="D10" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E10" s="15" t="n"/>
       <c r="F10" s="15" t="n"/>
       <c r="G10" s="15" t="n"/>
       <c r="H10" s="15" t="n"/>
       <c r="I10" s="15" t="n"/>
-      <c r="J10" s="15" t="n"/>
+      <c r="J10" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K10" s="15" t="n"/>
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="15" t="n"/>
@@ -1099,14 +1121,12 @@
       <c r="V10" s="15" t="n"/>
       <c r="W10" s="15" t="n"/>
       <c r="X10" s="15" t="n"/>
-      <c r="Y10" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y10" s="15" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>AIブームに乗って注目の半導体銘柄で長期投資を狙うなら？【坂本慎太郎の街歩き投資ラボ】 (週プレNEWS)</t>
+          <t>AIブームに乗って注目の半導体銘柄で長期投資を狙うなら？【坂本慎太郎の街歩き投資ラボ】（週プレNEWS）</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
@@ -1115,13 +1135,17 @@
         </is>
       </c>
       <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
+      <c r="D11" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="11" t="n"/>
       <c r="G11" s="11" t="n"/>
       <c r="H11" s="11" t="n"/>
       <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="n"/>
+      <c r="J11" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="K11" s="11" t="n"/>
       <c r="L11" s="11" t="n"/>
       <c r="M11" s="11" t="n"/>
@@ -1136,14 +1160,12 @@
       <c r="V11" s="11" t="n"/>
       <c r="W11" s="11" t="n"/>
       <c r="X11" s="11" t="n"/>
-      <c r="Y11" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>AIブームに乗って注目の半導体銘柄で長期投資を狙うなら？【坂本慎太郎の街歩き投資ラボ】（週プレNEWS）</t>
+          <t>【後場の投資戦略】AI・半導体関連株中心に利食い売り優勢</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -1152,13 +1174,17 @@
         </is>
       </c>
       <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
+      <c r="D12" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E12" s="15" t="n"/>
       <c r="F12" s="15" t="n"/>
       <c r="G12" s="15" t="n"/>
       <c r="H12" s="15" t="n"/>
       <c r="I12" s="15" t="n"/>
-      <c r="J12" s="15" t="n"/>
+      <c r="J12" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K12" s="15" t="n"/>
       <c r="L12" s="15" t="n"/>
       <c r="M12" s="15" t="n"/>
@@ -1173,14 +1199,12 @@
       <c r="V12" s="15" t="n"/>
       <c r="W12" s="15" t="n"/>
       <c r="X12" s="15" t="n"/>
-      <c r="Y12" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y12" s="15" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>【後場の投資戦略】AI・半導体関連株中心に利食い売り優勢</t>
+          <t>米、半導体装置の対中輸出規制 出荷停止要請と報道（共同通信）</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -1188,12 +1212,16 @@
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n"/>
+      <c r="C13" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="D13" s="11" t="n"/>
       <c r="E13" s="11" t="n"/>
       <c r="F13" s="11" t="n"/>
       <c r="G13" s="11" t="n"/>
-      <c r="H13" s="11" t="n"/>
+      <c r="H13" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="I13" s="11" t="n"/>
       <c r="J13" s="11" t="n"/>
       <c r="K13" s="11" t="n"/>
@@ -1204,20 +1232,20 @@
       <c r="P13" s="11" t="n"/>
       <c r="Q13" s="11" t="n"/>
       <c r="R13" s="11" t="n"/>
-      <c r="S13" s="11" t="n"/>
+      <c r="S13" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T13" s="11" t="n"/>
       <c r="U13" s="11" t="n"/>
       <c r="V13" s="11" t="n"/>
       <c r="W13" s="11" t="n"/>
       <c r="X13" s="11" t="n"/>
-      <c r="Y13" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>米、半導体装置の対中輸出規制 出荷停止要請と報道（共同通信）</t>
+          <t>3億ドル規模の新市場創出狙う…リガクが半導体検査装置を進化、米オントゥと提携</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -1226,7 +1254,9 @@
         </is>
       </c>
       <c r="C14" s="15" t="n"/>
-      <c r="D14" s="15" t="n"/>
+      <c r="D14" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E14" s="15" t="n"/>
       <c r="F14" s="15" t="n"/>
       <c r="G14" s="15" t="n"/>
@@ -1241,20 +1271,20 @@
       <c r="P14" s="15" t="n"/>
       <c r="Q14" s="15" t="n"/>
       <c r="R14" s="15" t="n"/>
-      <c r="S14" s="15" t="n"/>
+      <c r="S14" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T14" s="15" t="n"/>
       <c r="U14" s="15" t="n"/>
       <c r="V14" s="15" t="n"/>
       <c r="W14" s="15" t="n"/>
       <c r="X14" s="15" t="n"/>
-      <c r="Y14" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>3億ドル規模の新市場創出狙う…リガクが半導体検査装置を進化、米オントゥと提携</t>
+          <t>リガク、半導体検査装置を進化 米オントゥと提携</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -1263,7 +1293,9 @@
         </is>
       </c>
       <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
+      <c r="D15" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E15" s="11" t="n"/>
       <c r="F15" s="11" t="n"/>
       <c r="G15" s="11" t="n"/>
@@ -1278,20 +1310,20 @@
       <c r="P15" s="11" t="n"/>
       <c r="Q15" s="11" t="n"/>
       <c r="R15" s="11" t="n"/>
-      <c r="S15" s="11" t="n"/>
+      <c r="S15" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T15" s="11" t="n"/>
       <c r="U15" s="11" t="n"/>
       <c r="V15" s="11" t="n"/>
       <c r="W15" s="11" t="n"/>
       <c r="X15" s="11" t="n"/>
-      <c r="Y15" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>リガク、半導体検査装置を進化 米オントゥと提携</t>
+          <t>半導体検査装置 半導体テスタでは世界第１位の「アドバンテスト」 2026年3月期決算を発表 売上高１兆円突破！ 時価総額が一時２３兆円超え！</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -1300,7 +1332,9 @@
         </is>
       </c>
       <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
+      <c r="D16" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E16" s="15" t="n"/>
       <c r="F16" s="15" t="n"/>
       <c r="G16" s="15" t="n"/>
@@ -1315,20 +1349,22 @@
       <c r="P16" s="15" t="n"/>
       <c r="Q16" s="15" t="n"/>
       <c r="R16" s="15" t="n"/>
-      <c r="S16" s="15" t="n"/>
+      <c r="S16" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T16" s="15" t="n"/>
       <c r="U16" s="15" t="n"/>
       <c r="V16" s="15" t="n"/>
       <c r="W16" s="15" t="n"/>
-      <c r="X16" s="15" t="n"/>
-      <c r="Y16" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="X16" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y16" s="15" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>半導体検査装置 半導体テスタでは世界第１位の「アドバンテスト」 2026年3月期決算を発表 売上高１兆円突破！ 時価総額が一時２３兆円超え！</t>
+          <t>サーバーはもういらない？ 日立の「エッジAI半導体」が導く産業DXの完成形。半導体検査を1枚の画像で完遂、高速化とコスト低減を同時に実現</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -1337,13 +1373,17 @@
         </is>
       </c>
       <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
+      <c r="D17" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="11" t="n"/>
       <c r="H17" s="11" t="n"/>
       <c r="I17" s="11" t="n"/>
-      <c r="J17" s="11" t="n"/>
+      <c r="J17" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" s="11" t="n"/>
       <c r="L17" s="11" t="n"/>
       <c r="M17" s="11" t="n"/>
@@ -1358,23 +1398,23 @@
       <c r="V17" s="11" t="n"/>
       <c r="W17" s="11" t="n"/>
       <c r="X17" s="11" t="n"/>
-      <c r="Y17" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>サーバーはもういらない？ 日立の「エッジAI半導体」が導く産業DXの完成形。半導体検査を1枚の画像で完遂、高速化とコスト低減を同時に実現</t>
+          <t>半導体製造装置大手、韓国の売上比率が拡大</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="C18" s="15" t="n"/>
-      <c r="D18" s="15" t="n"/>
+      <c r="D18" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E18" s="15" t="n"/>
       <c r="F18" s="15" t="n"/>
       <c r="G18" s="15" t="n"/>
@@ -1389,20 +1429,20 @@
       <c r="P18" s="15" t="n"/>
       <c r="Q18" s="15" t="n"/>
       <c r="R18" s="15" t="n"/>
-      <c r="S18" s="15" t="n"/>
+      <c r="S18" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T18" s="15" t="n"/>
       <c r="U18" s="15" t="n"/>
       <c r="V18" s="15" t="n"/>
       <c r="W18" s="15" t="n"/>
       <c r="X18" s="15" t="n"/>
-      <c r="Y18" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y18" s="15" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>自動車用半導体市場：コンポーネント別、用途別、車種別、エンドユーザー別-2026年～2032年の世界市場予測</t>
+          <t>［新連載］半導体製造装置SCREEN、TSMCも頼る個別化・効率化</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -1411,7 +1451,9 @@
         </is>
       </c>
       <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
+      <c r="D19" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E19" s="11" t="n"/>
       <c r="F19" s="11" t="n"/>
       <c r="G19" s="11" t="n"/>
@@ -1426,20 +1468,20 @@
       <c r="P19" s="11" t="n"/>
       <c r="Q19" s="11" t="n"/>
       <c r="R19" s="11" t="n"/>
-      <c r="S19" s="11" t="n"/>
+      <c r="S19" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T19" s="11" t="n"/>
       <c r="U19" s="11" t="n"/>
       <c r="V19" s="11" t="n"/>
       <c r="W19" s="11" t="n"/>
       <c r="X19" s="11" t="n"/>
-      <c r="Y19" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>日経平均は続伸、最高値更新 米ＡＩ・半導体株高が支援</t>
+          <t>OKI、次世代AI半導体の検査装置向け180層・板厚15mmのPCB技術を確立</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -1448,13 +1490,17 @@
         </is>
       </c>
       <c r="C20" s="15" t="n"/>
-      <c r="D20" s="15" t="n"/>
+      <c r="D20" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E20" s="15" t="n"/>
       <c r="F20" s="15" t="n"/>
       <c r="G20" s="15" t="n"/>
       <c r="H20" s="15" t="n"/>
       <c r="I20" s="15" t="n"/>
-      <c r="J20" s="15" t="n"/>
+      <c r="J20" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="15" t="n"/>
       <c r="L20" s="15" t="n"/>
       <c r="M20" s="15" t="n"/>
@@ -1463,29 +1509,31 @@
       <c r="P20" s="15" t="n"/>
       <c r="Q20" s="15" t="n"/>
       <c r="R20" s="15" t="n"/>
-      <c r="S20" s="15" t="n"/>
+      <c r="S20" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T20" s="15" t="n"/>
       <c r="U20" s="15" t="n"/>
       <c r="V20" s="15" t="n"/>
       <c r="W20" s="15" t="n"/>
       <c r="X20" s="15" t="n"/>
-      <c r="Y20" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y20" s="15" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>半導体製造装置大手、韓国の売上比率が拡大</t>
+          <t>一時、株価6万円到達の背景 ～半導体価格の爆発～ | 熊野 英生 | 第一ライフ資産運用経済研究所</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
+      <c r="D21" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E21" s="11" t="n"/>
       <c r="F21" s="11" t="n"/>
       <c r="G21" s="11" t="n"/>
@@ -1505,24 +1553,26 @@
       <c r="U21" s="11" t="n"/>
       <c r="V21" s="11" t="n"/>
       <c r="W21" s="11" t="n"/>
-      <c r="X21" s="11" t="n"/>
-      <c r="Y21" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="X21" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>［新連載］半導体製造装置SCREEN、TSMCも頼る個別化・効率化</t>
+          <t>電子部品スクリーン印刷機の世界市場（2026年～2032年）、市場規模（カラー印刷、モノクロ印刷）・分析レポートを発表</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="C22" s="15" t="n"/>
-      <c r="D22" s="15" t="n"/>
+      <c r="D22" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E22" s="15" t="n"/>
       <c r="F22" s="15" t="n"/>
       <c r="G22" s="15" t="n"/>
@@ -1550,16 +1600,18 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>OKI、次世代AI半導体の検査装置向け180層・板厚15mmのPCB技術を確立</t>
+          <t>半導体製造装置SCREENHD、営業利益率10年で3倍 独自性と生産性を両立</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
+      <c r="D23" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E23" s="11" t="n"/>
       <c r="F23" s="11" t="n"/>
       <c r="G23" s="11" t="n"/>
@@ -1574,35 +1626,41 @@
       <c r="P23" s="11" t="n"/>
       <c r="Q23" s="11" t="n"/>
       <c r="R23" s="11" t="n"/>
-      <c r="S23" s="11" t="n"/>
+      <c r="S23" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T23" s="11" t="n"/>
       <c r="U23" s="11" t="n"/>
       <c r="V23" s="11" t="n"/>
       <c r="W23" s="11" t="n"/>
-      <c r="X23" s="11" t="n"/>
-      <c r="Y23" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="X23" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>日経平均が一時6万円！好業績・株価上昇期待の11銘柄</t>
+          <t>日本の半導体株、AI投資堅調で復調鮮明－成長期待のマネー集める</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
+      <c r="D24" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E24" s="15" t="n"/>
       <c r="F24" s="15" t="n"/>
       <c r="G24" s="15" t="n"/>
       <c r="H24" s="15" t="n"/>
       <c r="I24" s="15" t="n"/>
-      <c r="J24" s="15" t="n"/>
+      <c r="J24" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K24" s="15" t="n"/>
       <c r="L24" s="15" t="n"/>
       <c r="M24" s="15" t="n"/>
@@ -1617,29 +1675,31 @@
       <c r="V24" s="15" t="n"/>
       <c r="W24" s="15" t="n"/>
       <c r="X24" s="15" t="n"/>
-      <c r="Y24" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y24" s="15" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>電子部品スクリーン印刷機の世界市場（2026年～2032年）、市場規模（カラー印刷、モノクロ印刷）・分析レポートを発表</t>
+          <t>日本の半導体株、AI投資堅調で復調鮮明－成長期待のマネー集める（Bloomberg）</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="C25" s="11" t="n"/>
-      <c r="D25" s="11" t="n"/>
+      <c r="D25" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E25" s="11" t="n"/>
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
       <c r="H25" s="11" t="n"/>
       <c r="I25" s="11" t="n"/>
-      <c r="J25" s="11" t="n"/>
+      <c r="J25" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="K25" s="11" t="n"/>
       <c r="L25" s="11" t="n"/>
       <c r="M25" s="11" t="n"/>
@@ -1654,23 +1714,23 @@
       <c r="V25" s="11" t="n"/>
       <c r="W25" s="11" t="n"/>
       <c r="X25" s="11" t="n"/>
-      <c r="Y25" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>半導体製造装置SCREENHD、営業利益率10年で3倍 独自性と生産性を両立</t>
+          <t>TOTOKU、年度内に高導電性の半導体検査針量産化目指す（鉄鋼新聞）</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="C26" s="15" t="n"/>
-      <c r="D26" s="15" t="n"/>
+      <c r="D26" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E26" s="15" t="n"/>
       <c r="F26" s="15" t="n"/>
       <c r="G26" s="15" t="n"/>
@@ -1698,7 +1758,7 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>編集者の視点「半導体市場の膨張、CPU・メモリーけん引」</t>
+          <t>半導体バックエンド計測・検査装置の世界市場（2026年～2032年）、市場規模（計測・検査プロセス装置、欠陥検出プロセス装置、その他）・分析レポートを発表</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -1707,7 +1767,9 @@
         </is>
       </c>
       <c r="C27" s="11" t="n"/>
-      <c r="D27" s="11" t="n"/>
+      <c r="D27" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E27" s="11" t="n"/>
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="11" t="n"/>
@@ -1722,20 +1784,20 @@
       <c r="P27" s="11" t="n"/>
       <c r="Q27" s="11" t="n"/>
       <c r="R27" s="11" t="n"/>
-      <c r="S27" s="11" t="n"/>
+      <c r="S27" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T27" s="11" t="n"/>
       <c r="U27" s="11" t="n"/>
       <c r="V27" s="11" t="n"/>
       <c r="W27" s="11" t="n"/>
       <c r="X27" s="11" t="n"/>
-      <c r="Y27" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>車載半導体市場、2026年は25％増へ パワー半導体とマイコンが堅調 米ガートナー調査</t>
+          <t>半導体フロントエンド計測・検査装置の世界市場（2026年～2032年）、市場規模（計測・検査プロセス装置、欠陥検出プロセス装置、その他）・分析レポートを発表</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -1744,7 +1806,9 @@
         </is>
       </c>
       <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
+      <c r="D28" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E28" s="15" t="n"/>
       <c r="F28" s="15" t="n"/>
       <c r="G28" s="15" t="n"/>
@@ -1759,20 +1823,20 @@
       <c r="P28" s="15" t="n"/>
       <c r="Q28" s="15" t="n"/>
       <c r="R28" s="15" t="n"/>
-      <c r="S28" s="15" t="n"/>
+      <c r="S28" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T28" s="15" t="n"/>
       <c r="U28" s="15" t="n"/>
       <c r="V28" s="15" t="n"/>
       <c r="W28" s="15" t="n"/>
       <c r="X28" s="15" t="n"/>
-      <c r="Y28" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y28" s="15" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>日本の半導体株、AI投資堅調で復調鮮明－成長期待のマネー集める</t>
+          <t>シーシーエス、4/23に半導体検査・計測の工程効率化をテーマにWEBセミナーを開催</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
@@ -1781,7 +1845,9 @@
         </is>
       </c>
       <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
+      <c r="D29" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E29" s="11" t="n"/>
       <c r="F29" s="11" t="n"/>
       <c r="G29" s="11" t="n"/>
@@ -1809,16 +1875,18 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>日本の半導体株、AI投資堅調で復調鮮明－成長期待のマネー集める（Bloomberg）</t>
+          <t>日経平均が初の6万円、ＡＩ・半導体株がけん引 「Ｋ字相場」の側面も</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="C30" s="15" t="n"/>
-      <c r="D30" s="15" t="n"/>
+      <c r="D30" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E30" s="15" t="n"/>
       <c r="F30" s="15" t="n"/>
       <c r="G30" s="15" t="n"/>
@@ -1846,16 +1914,18 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>日本の半導体株、AI投資堅調で復調鮮明－成長期待のマネー集める フォトギャラリー | TBS CROSS DIG with Bloomberg</t>
+          <t>ＴＳＭＣ、ＡＳＭＬ高額新装置なしで小型・高速チップ製造へ</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="C31" s="11" t="n"/>
-      <c r="D31" s="11" t="n"/>
+      <c r="D31" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E31" s="11" t="n"/>
       <c r="F31" s="11" t="n"/>
       <c r="G31" s="11" t="n"/>
@@ -1883,16 +1953,18 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>TOTOKU、年度内に高導電性の半導体検査針量産化目指す（鉄鋼新聞）</t>
+          <t>コニカミノルタ、東京サイト八王子で半導体検査装置向け光学コンポーネントのガラスレンズの研磨工程を立ち上げ稼働開始</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
+      <c r="D32" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E32" s="15" t="n"/>
       <c r="F32" s="15" t="n"/>
       <c r="G32" s="15" t="n"/>
@@ -1907,29 +1979,31 @@
       <c r="P32" s="15" t="n"/>
       <c r="Q32" s="15" t="n"/>
       <c r="R32" s="15" t="n"/>
-      <c r="S32" s="15" t="n"/>
+      <c r="S32" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T32" s="15" t="n"/>
       <c r="U32" s="15" t="n"/>
       <c r="V32" s="15" t="n"/>
       <c r="W32" s="15" t="n"/>
       <c r="X32" s="15" t="n"/>
-      <c r="Y32" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y32" s="15" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>半導体バックエンド計測・検査装置の世界市場（2026年～2032年）、市場規模（計測・検査プロセス装置、欠陥検出プロセス装置、その他）・分析レポートを発表</t>
+          <t>2026年半導体市場規模は過去最高へ？スーパーサイクルと今後の見通しを解説</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
+      <c r="D33" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E33" s="11" t="n"/>
       <c r="F33" s="11" t="n"/>
       <c r="G33" s="11" t="n"/>
@@ -1957,16 +2031,18 @@
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>半導体フロントエンド計測・検査装置の世界市場（2026年～2032年）、市場規模（計測・検査プロセス装置、欠陥検出プロセス装置、その他）・分析レポートを発表</t>
+          <t>半導体製造装置用高性能セラミックス業界ランキング2026：売上、シェア、企業規模による分析</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
+      <c r="D34" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E34" s="15" t="n"/>
       <c r="F34" s="15" t="n"/>
       <c r="G34" s="15" t="n"/>
@@ -1981,29 +2057,31 @@
       <c r="P34" s="15" t="n"/>
       <c r="Q34" s="15" t="n"/>
       <c r="R34" s="15" t="n"/>
-      <c r="S34" s="15" t="n"/>
+      <c r="S34" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T34" s="15" t="n"/>
       <c r="U34" s="15" t="n"/>
       <c r="V34" s="15" t="n"/>
       <c r="W34" s="15" t="n"/>
       <c r="X34" s="15" t="n"/>
-      <c r="Y34" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y34" s="15" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>シーシーエス、4/23に半導体検査・計測の工程効率化をテーマにWEBセミナーを開催</t>
+          <t>化合物半導体市場規模・シェア・グローバルレポート2034</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C35" s="11" t="n"/>
-      <c r="D35" s="11" t="n"/>
+      <c r="D35" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E35" s="11" t="n"/>
       <c r="F35" s="11" t="n"/>
       <c r="G35" s="11" t="n"/>
@@ -2031,16 +2109,18 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>2026年の半導体市場1.3兆ドル予測の裏側、AI偏重とメモリの高騰が生む市場の二極化 | TECH+（テックプラス）</t>
+          <t>自動車用半導体市場規模、シェア及び成長予測 [2024-2033年]</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C36" s="15" t="n"/>
-      <c r="D36" s="15" t="n"/>
+      <c r="D36" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E36" s="15" t="n"/>
       <c r="F36" s="15" t="n"/>
       <c r="G36" s="15" t="n"/>
@@ -2068,16 +2148,18 @@
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>日経平均が初の6万円、ＡＩ・半導体株がけん引 「Ｋ字相場」の側面も</t>
+          <t>RF半導体市場規模、シェア |業界レポート [2032]</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C37" s="11" t="n"/>
-      <c r="D37" s="11" t="n"/>
+      <c r="D37" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E37" s="11" t="n"/>
       <c r="F37" s="11" t="n"/>
       <c r="G37" s="11" t="n"/>
@@ -2105,16 +2187,18 @@
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>ＴＳＭＣ、ＡＳＭＬ高額新装置なしで小型・高速チップ製造へ</t>
+          <t>電子機器製造サービス市場規模、予測【2034年】</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C38" s="15" t="n"/>
-      <c r="D38" s="15" t="n"/>
+      <c r="D38" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E38" s="15" t="n"/>
       <c r="F38" s="15" t="n"/>
       <c r="G38" s="15" t="n"/>
@@ -2142,16 +2226,18 @@
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>コニカミノルタ、東京サイト八王子で半導体検査装置向け光学コンポーネントのガラスレンズの研磨工程を立ち上げ稼働開始</t>
+          <t>コンシューマーエレクトロニクスの市場規模、シェア、傾向、成長、2034</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C39" s="11" t="n"/>
-      <c r="D39" s="11" t="n"/>
+      <c r="D39" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E39" s="11" t="n"/>
       <c r="F39" s="11" t="n"/>
       <c r="G39" s="11" t="n"/>
@@ -2179,16 +2265,18 @@
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>台湾、力強い成長局面へ：急成長するAI・半導体市場と人材・供給制約への対応が鍵に</t>
+          <t>半導体欠陥検査装置市場規模 [2034年]</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C40" s="15" t="n"/>
-      <c r="D40" s="15" t="n"/>
+      <c r="D40" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E40" s="15" t="n"/>
       <c r="F40" s="15" t="n"/>
       <c r="G40" s="15" t="n"/>
@@ -2203,35 +2291,39 @@
       <c r="P40" s="15" t="n"/>
       <c r="Q40" s="15" t="n"/>
       <c r="R40" s="15" t="n"/>
-      <c r="S40" s="15" t="n"/>
+      <c r="S40" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T40" s="15" t="n"/>
       <c r="U40" s="15" t="n"/>
       <c r="V40" s="15" t="n"/>
       <c r="W40" s="15" t="n"/>
       <c r="X40" s="15" t="n"/>
-      <c r="Y40" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y40" s="15" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>2026年半導体市場規模は過去最高へ？スーパーサイクルと今後の見通しを解説</t>
+          <t>今年1兆ドル突破へ、世界半導体市場の現在地 AI需要が招く「供給網の再編」と高騰する部材コスト（小久保重信） - エキスパート</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="C41" s="11" t="n"/>
-      <c r="D41" s="11" t="n"/>
+      <c r="D41" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E41" s="11" t="n"/>
       <c r="F41" s="11" t="n"/>
       <c r="G41" s="11" t="n"/>
       <c r="H41" s="11" t="n"/>
       <c r="I41" s="11" t="n"/>
-      <c r="J41" s="11" t="n"/>
+      <c r="J41" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="K41" s="11" t="n"/>
       <c r="L41" s="11" t="n"/>
       <c r="M41" s="11" t="n"/>
@@ -2246,23 +2338,23 @@
       <c r="V41" s="11" t="n"/>
       <c r="W41" s="11" t="n"/>
       <c r="X41" s="11" t="n"/>
-      <c r="Y41" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>半導体製造装置用高性能セラミックス業界ランキング2026：売上、シェア、企業規模による分析</t>
+          <t>アメリカの半導体検査装置メーカー｢エア･テスト･システムズ｣､売上高が44%減でも受注は6倍に</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="C42" s="15" t="n"/>
-      <c r="D42" s="15" t="n"/>
+      <c r="D42" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E42" s="15" t="n"/>
       <c r="F42" s="15" t="n"/>
       <c r="G42" s="15" t="n"/>
@@ -2277,29 +2369,33 @@
       <c r="P42" s="15" t="n"/>
       <c r="Q42" s="15" t="n"/>
       <c r="R42" s="15" t="n"/>
-      <c r="S42" s="15" t="n"/>
+      <c r="S42" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T42" s="15" t="n"/>
       <c r="U42" s="15" t="n"/>
       <c r="V42" s="15" t="n"/>
       <c r="W42" s="15" t="n"/>
-      <c r="X42" s="15" t="n"/>
-      <c r="Y42" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="X42" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y42" s="15" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>化合物半導体市場規模・シェア・グローバルレポート2034</t>
+          <t>キオクシア、東京エレクトロン、レゾナック、ディスコ…半導体セクターは「日本株の中心」であり続けるのか？主役交代説や“序列の変化”も解説！</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="C43" s="11" t="n"/>
-      <c r="D43" s="11" t="n"/>
+      <c r="D43" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E43" s="11" t="n"/>
       <c r="F43" s="11" t="n"/>
       <c r="G43" s="11" t="n"/>
@@ -2314,35 +2410,39 @@
       <c r="P43" s="11" t="n"/>
       <c r="Q43" s="11" t="n"/>
       <c r="R43" s="11" t="n"/>
-      <c r="S43" s="11" t="n"/>
+      <c r="S43" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T43" s="11" t="n"/>
       <c r="U43" s="11" t="n"/>
       <c r="V43" s="11" t="n"/>
       <c r="W43" s="11" t="n"/>
       <c r="X43" s="11" t="n"/>
-      <c r="Y43" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>自動車用半導体市場規模、シェア及び成長予測 [2024-2033年]</t>
+          <t>オランダ半導体製造装置大手 AI需要旺盛で見通し引き上げ</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="C44" s="15" t="n"/>
-      <c r="D44" s="15" t="n"/>
+      <c r="D44" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E44" s="15" t="n"/>
       <c r="F44" s="15" t="n"/>
       <c r="G44" s="15" t="n"/>
       <c r="H44" s="15" t="n"/>
       <c r="I44" s="15" t="n"/>
-      <c r="J44" s="15" t="n"/>
+      <c r="J44" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K44" s="15" t="n"/>
       <c r="L44" s="15" t="n"/>
       <c r="M44" s="15" t="n"/>
@@ -2351,29 +2451,31 @@
       <c r="P44" s="15" t="n"/>
       <c r="Q44" s="15" t="n"/>
       <c r="R44" s="15" t="n"/>
-      <c r="S44" s="15" t="n"/>
+      <c r="S44" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T44" s="15" t="n"/>
       <c r="U44" s="15" t="n"/>
       <c r="V44" s="15" t="n"/>
       <c r="W44" s="15" t="n"/>
       <c r="X44" s="15" t="n"/>
-      <c r="Y44" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y44" s="15" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>GaNおよびSiCパワー半導体市場規模、成長、2034年までの予測</t>
+          <t>世界の半導体の計測と検査メーカー分析：市場シェア、販売動向、価格変動2026</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="C45" s="11" t="n"/>
-      <c r="D45" s="11" t="n"/>
+      <c r="D45" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E45" s="11" t="n"/>
       <c r="F45" s="11" t="n"/>
       <c r="G45" s="11" t="n"/>
@@ -2401,16 +2503,18 @@
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>日本の半導体市場規模、2034年までに632億米ドルに到達――年平均成長率（CAGR）4.40%で拡大</t>
+          <t>先端半導体の需要が好調｢TSMC最新決算｣の中身。業績見通しを上方修正､通期で30%増収への写真一覧</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C46" s="15" t="n"/>
-      <c r="D46" s="15" t="n"/>
+      <c r="D46" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E46" s="15" t="n"/>
       <c r="F46" s="15" t="n"/>
       <c r="G46" s="15" t="n"/>
@@ -2430,24 +2534,26 @@
       <c r="U46" s="15" t="n"/>
       <c r="V46" s="15" t="n"/>
       <c r="W46" s="15" t="n"/>
-      <c r="X46" s="15" t="n"/>
-      <c r="Y46" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="X46" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y46" s="15" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>RF半導体市場規模、シェア |業界レポート [2032]</t>
+          <t>半導体製造装置ＡＳＭＬ、ＡＩ需要堅調で売上高見通し引き上げ</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C47" s="11" t="n"/>
-      <c r="D47" s="11" t="n"/>
+      <c r="D47" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E47" s="11" t="n"/>
       <c r="F47" s="11" t="n"/>
       <c r="G47" s="11" t="n"/>
@@ -2462,29 +2568,33 @@
       <c r="P47" s="11" t="n"/>
       <c r="Q47" s="11" t="n"/>
       <c r="R47" s="11" t="n"/>
-      <c r="S47" s="11" t="n"/>
+      <c r="S47" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T47" s="11" t="n"/>
       <c r="U47" s="11" t="n"/>
       <c r="V47" s="11" t="n"/>
       <c r="W47" s="11" t="n"/>
-      <c r="X47" s="11" t="n"/>
-      <c r="Y47" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="X47" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>ワイドバンドギャップ半導体市場サイズ、共有[2034]</t>
+          <t>オランダ半導体装置大手が業績予想上方修正</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C48" s="15" t="n"/>
-      <c r="D48" s="15" t="n"/>
+      <c r="D48" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E48" s="15" t="n"/>
       <c r="F48" s="15" t="n"/>
       <c r="G48" s="15" t="n"/>
@@ -2499,29 +2609,33 @@
       <c r="P48" s="15" t="n"/>
       <c r="Q48" s="15" t="n"/>
       <c r="R48" s="15" t="n"/>
-      <c r="S48" s="15" t="n"/>
+      <c r="S48" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T48" s="15" t="n"/>
       <c r="U48" s="15" t="n"/>
       <c r="V48" s="15" t="n"/>
       <c r="W48" s="15" t="n"/>
-      <c r="X48" s="15" t="n"/>
-      <c r="Y48" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="X48" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y48" s="15" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>電子機器製造サービス市場規模、予測【2034年】</t>
+          <t>オランダ半導体装置大手が業績予想上方修正｜全国のニュース｜Web東奥</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C49" s="11" t="n"/>
-      <c r="D49" s="11" t="n"/>
+      <c r="D49" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E49" s="11" t="n"/>
       <c r="F49" s="11" t="n"/>
       <c r="G49" s="11" t="n"/>
@@ -2536,29 +2650,33 @@
       <c r="P49" s="11" t="n"/>
       <c r="Q49" s="11" t="n"/>
       <c r="R49" s="11" t="n"/>
-      <c r="S49" s="11" t="n"/>
+      <c r="S49" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T49" s="11" t="n"/>
       <c r="U49" s="11" t="n"/>
       <c r="V49" s="11" t="n"/>
       <c r="W49" s="11" t="n"/>
-      <c r="X49" s="11" t="n"/>
-      <c r="Y49" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="X49" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>コンシューマーエレクトロニクスの市場規模、シェア、傾向、成長、2034</t>
+          <t>2026年半導体関連銘柄の本命は？日本の製造装置株が強い理由を徹底分析</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C50" s="15" t="n"/>
-      <c r="D50" s="15" t="n"/>
+      <c r="D50" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E50" s="15" t="n"/>
       <c r="F50" s="15" t="n"/>
       <c r="G50" s="15" t="n"/>
@@ -2573,29 +2691,31 @@
       <c r="P50" s="15" t="n"/>
       <c r="Q50" s="15" t="n"/>
       <c r="R50" s="15" t="n"/>
-      <c r="S50" s="15" t="n"/>
+      <c r="S50" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T50" s="15" t="n"/>
       <c r="U50" s="15" t="n"/>
       <c r="V50" s="15" t="n"/>
       <c r="W50" s="15" t="n"/>
       <c r="X50" s="15" t="n"/>
-      <c r="Y50" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y50" s="15" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>半導体欠陥検査装置市場規模 [2034年]</t>
+          <t>半導体製造装置の蘭ＡＳＭＬ、ＡＩ 需要堅調で売上高見通し上げ</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C51" s="11" t="n"/>
-      <c r="D51" s="11" t="n"/>
+      <c r="D51" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E51" s="11" t="n"/>
       <c r="F51" s="11" t="n"/>
       <c r="G51" s="11" t="n"/>
@@ -2610,29 +2730,33 @@
       <c r="P51" s="11" t="n"/>
       <c r="Q51" s="11" t="n"/>
       <c r="R51" s="11" t="n"/>
-      <c r="S51" s="11" t="n"/>
+      <c r="S51" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T51" s="11" t="n"/>
       <c r="U51" s="11" t="n"/>
       <c r="V51" s="11" t="n"/>
       <c r="W51" s="11" t="n"/>
-      <c r="X51" s="11" t="n"/>
-      <c r="Y51" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="X51" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>今年1兆ドル突破へ、世界半導体市場の現在地 AI需要が招く「供給網の再編」と高騰する部材コスト（小久保重信） - エキスパート</t>
+          <t>半導体製造装置ＡＳＭＬ、ＡＩ需要堅調で売上高見通し引き上げ(ロイター)</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C52" s="15" t="n"/>
-      <c r="D52" s="15" t="n"/>
+      <c r="D52" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E52" s="15" t="n"/>
       <c r="F52" s="15" t="n"/>
       <c r="G52" s="15" t="n"/>
@@ -2647,34 +2771,40 @@
       <c r="P52" s="15" t="n"/>
       <c r="Q52" s="15" t="n"/>
       <c r="R52" s="15" t="n"/>
-      <c r="S52" s="15" t="n"/>
+      <c r="S52" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T52" s="15" t="n"/>
       <c r="U52" s="15" t="n"/>
       <c r="V52" s="15" t="n"/>
       <c r="W52" s="15" t="n"/>
-      <c r="X52" s="15" t="n"/>
-      <c r="Y52" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="X52" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y52" s="15" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>アメリカの半導体検査装置メーカー｢エア･テスト･システムズ｣､売上高が44%減でも受注は6倍に</t>
+          <t>ニーズ高まる「パワー半導体」の組み立てや検査担う 三菱電機の新工場が完成 生産ライン集約で効率アップへ 福岡</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C53" s="11" t="n"/>
-      <c r="D53" s="11" t="n"/>
+      <c r="D53" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E53" s="11" t="n"/>
       <c r="F53" s="11" t="n"/>
       <c r="G53" s="11" t="n"/>
       <c r="H53" s="11" t="n"/>
-      <c r="I53" s="11" t="n"/>
+      <c r="I53" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="J53" s="11" t="n"/>
       <c r="K53" s="11" t="n"/>
       <c r="L53" s="11" t="n"/>
@@ -2685,32 +2815,36 @@
       <c r="Q53" s="11" t="n"/>
       <c r="R53" s="11" t="n"/>
       <c r="S53" s="11" t="n"/>
-      <c r="T53" s="11" t="n"/>
+      <c r="T53" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="U53" s="11" t="n"/>
       <c r="V53" s="11" t="n"/>
       <c r="W53" s="11" t="n"/>
       <c r="X53" s="11" t="n"/>
-      <c r="Y53" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>キオクシア、東京エレクトロン、レゾナック、ディスコ…半導体セクターは「日本株の中心」であり続けるのか？主役交代説や“序列の変化”も解説！</t>
+          <t>日本の半導体企業にも影響大か 米議会、対中輸出規制の新法案</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="C54" s="15" t="n"/>
-      <c r="D54" s="15" t="n"/>
+      <c r="D54" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E54" s="15" t="n"/>
       <c r="F54" s="15" t="n"/>
       <c r="G54" s="15" t="n"/>
-      <c r="H54" s="15" t="n"/>
+      <c r="H54" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="I54" s="15" t="n"/>
       <c r="J54" s="15" t="n"/>
       <c r="K54" s="15" t="n"/>
@@ -2727,23 +2861,23 @@
       <c r="V54" s="15" t="n"/>
       <c r="W54" s="15" t="n"/>
       <c r="X54" s="15" t="n"/>
-      <c r="Y54" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y54" s="15" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>オランダ半導体製造装置大手 AI需要旺盛で見通し引き上げ</t>
+          <t>デジタル時代の半導体製造装置需要の変遷</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="C55" s="11" t="n"/>
-      <c r="D55" s="11" t="n"/>
+      <c r="D55" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E55" s="11" t="n"/>
       <c r="F55" s="11" t="n"/>
       <c r="G55" s="11" t="n"/>
@@ -2758,29 +2892,31 @@
       <c r="P55" s="11" t="n"/>
       <c r="Q55" s="11" t="n"/>
       <c r="R55" s="11" t="n"/>
-      <c r="S55" s="11" t="n"/>
+      <c r="S55" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T55" s="11" t="n"/>
       <c r="U55" s="11" t="n"/>
       <c r="V55" s="11" t="n"/>
       <c r="W55" s="11" t="n"/>
       <c r="X55" s="11" t="n"/>
-      <c r="Y55" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>世界の半導体の計測と検査メーカー分析：市場シェア、販売動向、価格変動2026</t>
+          <t>「半導体製造装置」が５位、ＳＯＸ指数９連騰で初の９０００大台ライン突破＜注目テーマ＞</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="C56" s="15" t="n"/>
-      <c r="D56" s="15" t="n"/>
+      <c r="D56" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E56" s="15" t="n"/>
       <c r="F56" s="15" t="n"/>
       <c r="G56" s="15" t="n"/>
@@ -2795,29 +2931,31 @@
       <c r="P56" s="15" t="n"/>
       <c r="Q56" s="15" t="n"/>
       <c r="R56" s="15" t="n"/>
-      <c r="S56" s="15" t="n"/>
+      <c r="S56" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T56" s="15" t="n"/>
       <c r="U56" s="15" t="n"/>
       <c r="V56" s="15" t="n"/>
       <c r="W56" s="15" t="n"/>
       <c r="X56" s="15" t="n"/>
-      <c r="Y56" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y56" s="15" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>有機半導体市場：市場規模・シェア・予測（2035年まで）</t>
+          <t>半導体市場の規模、シェア、成長、予測 [2034]</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C57" s="11" t="n"/>
-      <c r="D57" s="11" t="n"/>
+      <c r="D57" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E57" s="11" t="n"/>
       <c r="F57" s="11" t="n"/>
       <c r="G57" s="11" t="n"/>
@@ -2845,16 +2983,18 @@
     <row r="58">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>先端半導体の需要が好調｢TSMC最新決算｣の中身。業績見通しを上方修正､通期で30%増収への写真一覧</t>
+          <t>半導体とその先へ</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C58" s="15" t="n"/>
-      <c r="D58" s="15" t="n"/>
+      <c r="D58" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E58" s="15" t="n"/>
       <c r="F58" s="15" t="n"/>
       <c r="G58" s="15" t="n"/>
@@ -2882,16 +3022,18 @@
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>半導体製造装置ＡＳＭＬ、ＡＩ需要堅調で売上高見通し引き上げ</t>
+          <t>日本の半導体市場規模、シェア、成長、2026-2034</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C59" s="11" t="n"/>
-      <c r="D59" s="11" t="n"/>
+      <c r="D59" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E59" s="11" t="n"/>
       <c r="F59" s="11" t="n"/>
       <c r="G59" s="11" t="n"/>
@@ -2919,16 +3061,18 @@
     <row r="60">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>オランダ半導体装置大手が業績予想上方修正</t>
+          <t>アナログ半導体市場サイズ、共有|成長レポート、2034</t>
         </is>
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C60" s="15" t="n"/>
-      <c r="D60" s="15" t="n"/>
+      <c r="D60" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E60" s="15" t="n"/>
       <c r="F60" s="15" t="n"/>
       <c r="G60" s="15" t="n"/>
@@ -2956,16 +3100,18 @@
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>オランダ半導体装置大手が業績予想上方修正｜全国のニュース｜Web東奥</t>
+          <t>フレキシブルエレクトロニクス市場規模、シェア、収益、2034年予測</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C61" s="11" t="n"/>
-      <c r="D61" s="11" t="n"/>
+      <c r="D61" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E61" s="11" t="n"/>
       <c r="F61" s="11" t="n"/>
       <c r="G61" s="11" t="n"/>
@@ -2993,16 +3139,18 @@
     <row r="62">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>2026年半導体関連銘柄の本命は？日本の製造装置株が強い理由を徹底分析</t>
+          <t>ポリシリコン市場規模、シェア、分析、業界見通し、2034年</t>
         </is>
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C62" s="15" t="n"/>
-      <c r="D62" s="15" t="n"/>
+      <c r="D62" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E62" s="15" t="n"/>
       <c r="F62" s="15" t="n"/>
       <c r="G62" s="15" t="n"/>
@@ -3030,16 +3178,18 @@
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>半導体製造装置の蘭ＡＳＭＬ、ＡＩ 需要堅調で売上高見通し上げ</t>
+          <t>半導体エッチング装置市場規模｜業界予測［2026-2034年］</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="C63" s="11" t="n"/>
-      <c r="D63" s="11" t="n"/>
+      <c r="D63" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E63" s="11" t="n"/>
       <c r="F63" s="11" t="n"/>
       <c r="G63" s="11" t="n"/>
@@ -3054,29 +3204,31 @@
       <c r="P63" s="11" t="n"/>
       <c r="Q63" s="11" t="n"/>
       <c r="R63" s="11" t="n"/>
-      <c r="S63" s="11" t="n"/>
+      <c r="S63" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T63" s="11" t="n"/>
       <c r="U63" s="11" t="n"/>
       <c r="V63" s="11" t="n"/>
       <c r="W63" s="11" t="n"/>
       <c r="X63" s="11" t="n"/>
-      <c r="Y63" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>半導体製造装置ＡＳＭＬ、ＡＩ需要堅調で売上高見通し引き上げ(ロイター)</t>
+          <t>荏原、半導体投資800億円超 3年で 研磨装置 シェア首位目指す</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="C64" s="15" t="n"/>
-      <c r="D64" s="15" t="n"/>
+      <c r="D64" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E64" s="15" t="n"/>
       <c r="F64" s="15" t="n"/>
       <c r="G64" s="15" t="n"/>
@@ -3104,22 +3256,26 @@
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>ニーズ高まる「パワー半導体」の組み立てや検査担う 三菱電機の新工場が完成 生産ライン集約で効率アップへ 福岡</t>
+          <t>半導体製造装置メーカーのプロセス開発領域にて初活用製造ライン改善ログを横断解析し“再現可能な生産性向上”を実現するAI基盤「AI IPGenius」</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="C65" s="11" t="n"/>
-      <c r="D65" s="11" t="n"/>
+      <c r="D65" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E65" s="11" t="n"/>
       <c r="F65" s="11" t="n"/>
       <c r="G65" s="11" t="n"/>
       <c r="H65" s="11" t="n"/>
       <c r="I65" s="11" t="n"/>
-      <c r="J65" s="11" t="n"/>
+      <c r="J65" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="K65" s="11" t="n"/>
       <c r="L65" s="11" t="n"/>
       <c r="M65" s="11" t="n"/>
@@ -3128,37 +3284,43 @@
       <c r="P65" s="11" t="n"/>
       <c r="Q65" s="11" t="n"/>
       <c r="R65" s="11" t="n"/>
-      <c r="S65" s="11" t="n"/>
+      <c r="S65" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T65" s="11" t="n"/>
       <c r="U65" s="11" t="n"/>
       <c r="V65" s="11" t="n"/>
       <c r="W65" s="11" t="n"/>
       <c r="X65" s="11" t="n"/>
-      <c r="Y65" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>日本の半導体企業にも影響大か 米議会、対中輸出規制の新法案</t>
+          <t>26年の半導体市場は64％成長で1.3兆ドルに NAND価格は234％上昇：非AI分野の需要は減退か先送りに</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="C66" s="15" t="n"/>
-      <c r="D66" s="15" t="n"/>
+      <c r="D66" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E66" s="15" t="n"/>
       <c r="F66" s="15" t="n"/>
       <c r="G66" s="15" t="n"/>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="15" t="n"/>
-      <c r="J66" s="15" t="n"/>
+      <c r="J66" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K66" s="15" t="n"/>
-      <c r="L66" s="15" t="n"/>
+      <c r="L66" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="M66" s="15" t="n"/>
       <c r="N66" s="15" t="n"/>
       <c r="O66" s="15" t="n"/>
@@ -3171,23 +3333,23 @@
       <c r="V66" s="15" t="n"/>
       <c r="W66" s="15" t="n"/>
       <c r="X66" s="15" t="n"/>
-      <c r="Y66" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y66" s="15" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>デジタル時代の半導体製造装置需要の変遷</t>
+          <t>半導体製造装置の世界販売、25年は15％増 日本も先端向けがけん引（電波新聞デジタル）</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="C67" s="11" t="n"/>
-      <c r="D67" s="11" t="n"/>
+      <c r="D67" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E67" s="11" t="n"/>
       <c r="F67" s="11" t="n"/>
       <c r="G67" s="11" t="n"/>
@@ -3202,35 +3364,39 @@
       <c r="P67" s="11" t="n"/>
       <c r="Q67" s="11" t="n"/>
       <c r="R67" s="11" t="n"/>
-      <c r="S67" s="11" t="n"/>
+      <c r="S67" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T67" s="11" t="n"/>
       <c r="U67" s="11" t="n"/>
       <c r="V67" s="11" t="n"/>
       <c r="W67" s="11" t="n"/>
       <c r="X67" s="11" t="n"/>
-      <c r="Y67" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>「半導体製造装置」が５位、ＳＯＸ指数９連騰で初の９０００大台ライン突破＜注目テーマ＞</t>
+          <t>テスラの巨大AI半導体工場、インテル参画 テラファブ「製造技術を刷新」</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="C68" s="15" t="n"/>
-      <c r="D68" s="15" t="n"/>
+      <c r="D68" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E68" s="15" t="n"/>
       <c r="F68" s="15" t="n"/>
       <c r="G68" s="15" t="n"/>
       <c r="H68" s="15" t="n"/>
       <c r="I68" s="15" t="n"/>
-      <c r="J68" s="15" t="n"/>
+      <c r="J68" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K68" s="15" t="n"/>
       <c r="L68" s="15" t="n"/>
       <c r="M68" s="15" t="n"/>
@@ -3245,23 +3411,23 @@
       <c r="V68" s="15" t="n"/>
       <c r="W68" s="15" t="n"/>
       <c r="X68" s="15" t="n"/>
-      <c r="Y68" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y68" s="15" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>半導体市場の規模、シェア、成長、予測 [2034]</t>
+          <t>続編：2026年日本の半導体工場の最新事情 | サイエンス リポート | TELESCOPE magazine</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C69" s="11" t="n"/>
-      <c r="D69" s="11" t="n"/>
+      <c r="D69" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E69" s="11" t="n"/>
       <c r="F69" s="11" t="n"/>
       <c r="G69" s="11" t="n"/>
@@ -3276,35 +3442,39 @@
       <c r="P69" s="11" t="n"/>
       <c r="Q69" s="11" t="n"/>
       <c r="R69" s="11" t="n"/>
-      <c r="S69" s="11" t="n"/>
+      <c r="S69" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T69" s="11" t="n"/>
       <c r="U69" s="11" t="n"/>
       <c r="V69" s="11" t="n"/>
       <c r="W69" s="11" t="n"/>
       <c r="X69" s="11" t="n"/>
-      <c r="Y69" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>半導体とその先へ</t>
+          <t>半導体装置、AI需要がサイクルの「谷」打ち消す</t>
         </is>
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C70" s="15" t="n"/>
-      <c r="D70" s="15" t="n"/>
+      <c r="D70" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E70" s="15" t="n"/>
       <c r="F70" s="15" t="n"/>
       <c r="G70" s="15" t="n"/>
       <c r="H70" s="15" t="n"/>
       <c r="I70" s="15" t="n"/>
-      <c r="J70" s="15" t="n"/>
+      <c r="J70" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K70" s="15" t="n"/>
       <c r="L70" s="15" t="n"/>
       <c r="M70" s="15" t="n"/>
@@ -3313,29 +3483,31 @@
       <c r="P70" s="15" t="n"/>
       <c r="Q70" s="15" t="n"/>
       <c r="R70" s="15" t="n"/>
-      <c r="S70" s="15" t="n"/>
+      <c r="S70" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T70" s="15" t="n"/>
       <c r="U70" s="15" t="n"/>
       <c r="V70" s="15" t="n"/>
       <c r="W70" s="15" t="n"/>
       <c r="X70" s="15" t="n"/>
-      <c r="Y70" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y70" s="15" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>日本の半導体市場規模、シェア、成長、2026-2034</t>
+          <t>エプソン、インクジェットで半導体製造 ラピダスに出資「連携深める」</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C71" s="11" t="n"/>
-      <c r="D71" s="11" t="n"/>
+      <c r="D71" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E71" s="11" t="n"/>
       <c r="F71" s="11" t="n"/>
       <c r="G71" s="11" t="n"/>
@@ -3363,16 +3535,18 @@
     <row r="72">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>アナログ半導体市場サイズ、共有|成長レポート、2034</t>
+          <t>半導体製造装置大手TOWA、「COMPANY® Talent Management」シリーズで国内外の人材データを一元化、客観的なデータに基づいた適材適所を実現 | 株式会社WHI Holdings</t>
         </is>
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="C72" s="15" t="n"/>
-      <c r="D72" s="15" t="n"/>
+      <c r="D72" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E72" s="15" t="n"/>
       <c r="F72" s="15" t="n"/>
       <c r="G72" s="15" t="n"/>
@@ -3387,29 +3561,31 @@
       <c r="P72" s="15" t="n"/>
       <c r="Q72" s="15" t="n"/>
       <c r="R72" s="15" t="n"/>
-      <c r="S72" s="15" t="n"/>
+      <c r="S72" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T72" s="15" t="n"/>
       <c r="U72" s="15" t="n"/>
       <c r="V72" s="15" t="n"/>
       <c r="W72" s="15" t="n"/>
       <c r="X72" s="15" t="n"/>
-      <c r="Y72" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>携帯電話用半導体市場規模・シェア |成長 [2034]</t>
+          <t>半導体製造装置大手TOWA、「COMPANY® Talent Management」シリーズで国内外の人材データを一元化、客観的なデータに基づいた適材適所を実現</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="C73" s="11" t="n"/>
-      <c r="D73" s="11" t="n"/>
+      <c r="D73" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E73" s="11" t="n"/>
       <c r="F73" s="11" t="n"/>
       <c r="G73" s="11" t="n"/>
@@ -3424,29 +3600,31 @@
       <c r="P73" s="11" t="n"/>
       <c r="Q73" s="11" t="n"/>
       <c r="R73" s="11" t="n"/>
-      <c r="S73" s="11" t="n"/>
+      <c r="S73" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T73" s="11" t="n"/>
       <c r="U73" s="11" t="n"/>
       <c r="V73" s="11" t="n"/>
       <c r="W73" s="11" t="n"/>
       <c r="X73" s="11" t="n"/>
-      <c r="Y73" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>光半導体市場規模、成長動向及びレポート [2026-2034年]</t>
+          <t>世界半導体市場は26年2月に大幅成長、日本のみ9カ月連続マイナスに：全体は前年比61.8％増</t>
         </is>
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C74" s="15" t="n"/>
-      <c r="D74" s="15" t="n"/>
+      <c r="D74" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E74" s="15" t="n"/>
       <c r="F74" s="15" t="n"/>
       <c r="G74" s="15" t="n"/>
@@ -3474,22 +3652,28 @@
     <row r="75">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>ディスクリート半導体市場規模、シェア、世界レポート、2034年</t>
+          <t>内閣府と経産省、第2回AI・半導体ワーキンググループ開催 バーティカルAIなどへの投資を議論</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C75" s="11" t="n"/>
-      <c r="D75" s="11" t="n"/>
+      <c r="D75" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E75" s="11" t="n"/>
       <c r="F75" s="11" t="n"/>
-      <c r="G75" s="11" t="n"/>
+      <c r="G75" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="H75" s="11" t="n"/>
       <c r="I75" s="11" t="n"/>
-      <c r="J75" s="11" t="n"/>
+      <c r="J75" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="K75" s="11" t="n"/>
       <c r="L75" s="11" t="n"/>
       <c r="M75" s="11" t="n"/>
@@ -3504,35 +3688,39 @@
       <c r="V75" s="11" t="n"/>
       <c r="W75" s="11" t="n"/>
       <c r="X75" s="11" t="n"/>
-      <c r="Y75" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>半導体リードフレーム市場サイズ、成長分析[2034]</t>
+          <t>AIを軸に日本にチャンス到来、データセンター投資、半導体材料が活発に</t>
         </is>
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C76" s="15" t="n"/>
-      <c r="D76" s="15" t="n"/>
+      <c r="D76" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E76" s="15" t="n"/>
       <c r="F76" s="15" t="n"/>
       <c r="G76" s="15" t="n"/>
       <c r="H76" s="15" t="n"/>
       <c r="I76" s="15" t="n"/>
-      <c r="J76" s="15" t="n"/>
+      <c r="J76" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K76" s="15" t="n"/>
       <c r="L76" s="15" t="n"/>
       <c r="M76" s="15" t="n"/>
       <c r="N76" s="15" t="n"/>
       <c r="O76" s="15" t="n"/>
-      <c r="P76" s="15" t="n"/>
+      <c r="P76" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="Q76" s="15" t="n"/>
       <c r="R76" s="15" t="n"/>
       <c r="S76" s="15" t="n"/>
@@ -3541,23 +3729,23 @@
       <c r="V76" s="15" t="n"/>
       <c r="W76" s="15" t="n"/>
       <c r="X76" s="15" t="n"/>
-      <c r="Y76" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y76" s="15" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>フレキシブルエレクトロニクス市場規模、シェア、収益、2034年予測</t>
+          <t>一般電子部品の日本市場（～2031年）、市場規模（能動部品、受動部品、電気機械部品）・分析レポートを発表</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C77" s="11" t="n"/>
-      <c r="D77" s="11" t="n"/>
+      <c r="D77" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E77" s="11" t="n"/>
       <c r="F77" s="11" t="n"/>
       <c r="G77" s="11" t="n"/>
@@ -3585,16 +3773,18 @@
     <row r="78">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>ポリシリコン市場規模、シェア、分析、業界見通し、2034年</t>
+          <t>堀場製作所は実は半導体の「ニッチトップ」企業！世界シェア6割を握る機器とは？創業家3代目が絶好調の受注環境を激白、問われるアクティビストへの対応力</t>
         </is>
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C78" s="15" t="n"/>
-      <c r="D78" s="15" t="n"/>
+      <c r="D78" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E78" s="15" t="n"/>
       <c r="F78" s="15" t="n"/>
       <c r="G78" s="15" t="n"/>
@@ -3622,16 +3812,18 @@
     <row r="79">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t>半導体エッチング装置市場規模｜業界予測［2026-2034年］</t>
+          <t>オプテックスグループ[6914]：シーシーエスが自動車・半導体検査ソリューションの展示会を東海地方のお客様向けに開催 2026年4月6日(適時開示) ：日経会社情報DIGITAL</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C79" s="11" t="n"/>
-      <c r="D79" s="11" t="n"/>
+      <c r="D79" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E79" s="11" t="n"/>
       <c r="F79" s="11" t="n"/>
       <c r="G79" s="11" t="n"/>
@@ -3659,16 +3851,18 @@
     <row r="80">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>アマゾン、「ＮＶＩＤＩＡの独走」と言われるＡＩ半導体市場に「自社チップ」で挑戦状 : 経済</t>
+          <t>半導体アセンブリおよびテストサービス市場規模[2028]</t>
         </is>
       </c>
       <c r="B80" s="14" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C80" s="15" t="n"/>
-      <c r="D80" s="15" t="n"/>
+      <c r="D80" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E80" s="15" t="n"/>
       <c r="F80" s="15" t="n"/>
       <c r="G80" s="15" t="n"/>
@@ -3696,16 +3890,18 @@
     <row r="81">
       <c r="A81" s="9" t="inlineStr">
         <is>
-          <t>荏原、半導体投資800億円超 3年で 研磨装置 シェア首位目指す</t>
+          <t>シーシーエスが自動車・半導体検査ソリューションの展示会を 東海地方のお客様向けに開催</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C81" s="11" t="n"/>
-      <c r="D81" s="11" t="n"/>
+      <c r="D81" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E81" s="11" t="n"/>
       <c r="F81" s="11" t="n"/>
       <c r="G81" s="11" t="n"/>
@@ -3733,20 +3929,24 @@
     <row r="82">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>半導体製造装置メーカーのプロセス開発領域にて初活用製造ライン改善ログを横断解析し“再現可能な生産性向上”を実現するAI基盤「AI IPGenius」</t>
+          <t>米議員グループ、対中半導体装置輸出の規制強化法案を公表</t>
         </is>
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="C82" s="15" t="n"/>
-      <c r="D82" s="15" t="n"/>
+      <c r="D82" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E82" s="15" t="n"/>
       <c r="F82" s="15" t="n"/>
       <c r="G82" s="15" t="n"/>
-      <c r="H82" s="15" t="n"/>
+      <c r="H82" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="I82" s="15" t="n"/>
       <c r="J82" s="15" t="n"/>
       <c r="K82" s="15" t="n"/>
@@ -3757,29 +3957,31 @@
       <c r="P82" s="15" t="n"/>
       <c r="Q82" s="15" t="n"/>
       <c r="R82" s="15" t="n"/>
-      <c r="S82" s="15" t="n"/>
+      <c r="S82" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="T82" s="15" t="n"/>
       <c r="U82" s="15" t="n"/>
       <c r="V82" s="15" t="n"/>
       <c r="W82" s="15" t="n"/>
       <c r="X82" s="15" t="n"/>
-      <c r="Y82" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y82" s="15" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>26年の半導体市場は64％成長で1.3兆ドルに NAND価格は234％上昇：非AI分野の需要は減退か先送りに</t>
+          <t>ロジック半導体の日本市場（～2031年）、市場規模（特殊用途ロジック、ディスプレイドライバ、汎用ロジック）・分析レポートを発表</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="C83" s="11" t="n"/>
-      <c r="D83" s="11" t="n"/>
+      <c r="D83" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E83" s="11" t="n"/>
       <c r="F83" s="11" t="n"/>
       <c r="G83" s="11" t="n"/>
@@ -3790,7 +3992,9 @@
       <c r="L83" s="11" t="n"/>
       <c r="M83" s="11" t="n"/>
       <c r="N83" s="11" t="n"/>
-      <c r="O83" s="11" t="n"/>
+      <c r="O83" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="P83" s="11" t="n"/>
       <c r="Q83" s="11" t="n"/>
       <c r="R83" s="11" t="n"/>
@@ -3800,29 +4004,33 @@
       <c r="V83" s="11" t="n"/>
       <c r="W83" s="11" t="n"/>
       <c r="X83" s="11" t="n"/>
-      <c r="Y83" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>半導体製造装置の世界販売、25年は15％増 日本も先端向けがけん引（電波新聞デジタル）</t>
+          <t>マイクロソフト、日本の AI 主導型成長に 1 兆 6000 億円を投資。AI インフラ、国家安全保障、人材育成を通じたさらなる国力強化を支援</t>
         </is>
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="C84" s="15" t="n"/>
-      <c r="D84" s="15" t="n"/>
+      <c r="D84" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E84" s="15" t="n"/>
       <c r="F84" s="15" t="n"/>
       <c r="G84" s="15" t="n"/>
-      <c r="H84" s="15" t="n"/>
+      <c r="H84" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="I84" s="15" t="n"/>
-      <c r="J84" s="15" t="n"/>
+      <c r="J84" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K84" s="15" t="n"/>
       <c r="L84" s="15" t="n"/>
       <c r="M84" s="15" t="n"/>
@@ -3837,23 +4045,23 @@
       <c r="V84" s="15" t="n"/>
       <c r="W84" s="15" t="n"/>
       <c r="X84" s="15" t="n"/>
-      <c r="Y84" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y84" s="15" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="inlineStr">
         <is>
-          <t>テスラの巨大AI半導体工場、インテル参画 テラファブ「製造技術を刷新」</t>
+          <t>2026年、27年とも300mm工場への設備投資は2桁成長～SEMI予測</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="C85" s="11" t="n"/>
-      <c r="D85" s="11" t="n"/>
+      <c r="D85" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E85" s="11" t="n"/>
       <c r="F85" s="11" t="n"/>
       <c r="G85" s="11" t="n"/>
@@ -3868,28 +4076,30 @@
       <c r="P85" s="11" t="n"/>
       <c r="Q85" s="11" t="n"/>
       <c r="R85" s="11" t="n"/>
-      <c r="S85" s="11" t="n"/>
+      <c r="S85" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T85" s="11" t="n"/>
       <c r="U85" s="11" t="n"/>
       <c r="V85" s="11" t="n"/>
       <c r="W85" s="11" t="n"/>
       <c r="X85" s="11" t="n"/>
-      <c r="Y85" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>続編：2026年日本の半導体工場の最新事情 | サイエンス リポート | TELESCOPE magazine</t>
+          <t>中国ＡＩ半導体市場、国内勢がシェア4割強 エヌビディア優位性縮小</t>
         </is>
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="C86" s="15" t="n"/>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C86" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="D86" s="15" t="n"/>
       <c r="E86" s="15" t="n"/>
       <c r="F86" s="15" t="n"/>
@@ -3918,16 +4128,18 @@
     <row r="87">
       <c r="A87" s="9" t="inlineStr">
         <is>
-          <t>半導体装置、AI需要がサイクルの「谷」打ち消す</t>
+          <t>競争激しい半導体市場へ…日本ガイシが4月から『NGK』に 社名変更の背景に“祖業からのシフトチェンジ”</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C87" s="11" t="n"/>
-      <c r="D87" s="11" t="n"/>
+      <c r="D87" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E87" s="11" t="n"/>
       <c r="F87" s="11" t="n"/>
       <c r="G87" s="11" t="n"/>
@@ -3955,22 +4167,26 @@
     <row r="88">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>エプソン、インクジェットで半導体製造 ラピダスに出資「連携深める」</t>
+          <t>世界の供給網に「ヘリウムショック」 MRI検査からAI半導体まで波及</t>
         </is>
       </c>
       <c r="B88" s="14" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C88" s="15" t="n"/>
-      <c r="D88" s="15" t="n"/>
+      <c r="D88" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E88" s="15" t="n"/>
       <c r="F88" s="15" t="n"/>
       <c r="G88" s="15" t="n"/>
       <c r="H88" s="15" t="n"/>
       <c r="I88" s="15" t="n"/>
-      <c r="J88" s="15" t="n"/>
+      <c r="J88" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="K88" s="15" t="n"/>
       <c r="L88" s="15" t="n"/>
       <c r="M88" s="15" t="n"/>
@@ -3985,23 +4201,23 @@
       <c r="V88" s="15" t="n"/>
       <c r="W88" s="15" t="n"/>
       <c r="X88" s="15" t="n"/>
-      <c r="Y88" s="16" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y88" s="15" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="inlineStr">
         <is>
-          <t>半導体製造装置大手TOWA、「COMPANY® Talent Management」シリーズで国内外の人材データを一元化、客観的なデータに基づいた適材適所を実現 | 株式会社WHI Holdings</t>
+          <t>アドテスト、ユーロ円建てＣＢ1000億円 半導体検査装置の生産能力増強</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C89" s="11" t="n"/>
-      <c r="D89" s="11" t="n"/>
+      <c r="D89" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E89" s="11" t="n"/>
       <c r="F89" s="11" t="n"/>
       <c r="G89" s="11" t="n"/>
@@ -4016,29 +4232,31 @@
       <c r="P89" s="11" t="n"/>
       <c r="Q89" s="11" t="n"/>
       <c r="R89" s="11" t="n"/>
-      <c r="S89" s="11" t="n"/>
+      <c r="S89" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T89" s="11" t="n"/>
       <c r="U89" s="11" t="n"/>
       <c r="V89" s="11" t="n"/>
       <c r="W89" s="11" t="n"/>
       <c r="X89" s="11" t="n"/>
-      <c r="Y89" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>半導体製造装置大手TOWA、「COMPANY® Talent Management」シリーズで国内外の人材データを一元化、客観的なデータに基づいた適材適所を実現</t>
+          <t>半導体製造は日本企業の技術が必須 業界マップで投資先探し</t>
         </is>
       </c>
       <c r="B90" s="14" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C90" s="15" t="n"/>
-      <c r="D90" s="15" t="n"/>
+      <c r="D90" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="E90" s="15" t="n"/>
       <c r="F90" s="15" t="n"/>
       <c r="G90" s="15" t="n"/>
@@ -4066,16 +4284,18 @@
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>旭有機材、宮崎県延岡市に新工場建設 半導体製造装置向けバルブ生産能力3倍へ 175億円投資</t>
+          <t>半導体ウェハ検査技術のPhoto electron Soul、約9億円の資金調達を完了</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C91" s="11" t="n"/>
-      <c r="D91" s="11" t="n"/>
+      <c r="D91" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="E91" s="11" t="n"/>
       <c r="F91" s="11" t="n"/>
       <c r="G91" s="11" t="n"/>
@@ -4090,681 +4310,15 @@
       <c r="P91" s="11" t="n"/>
       <c r="Q91" s="11" t="n"/>
       <c r="R91" s="11" t="n"/>
-      <c r="S91" s="11" t="n"/>
+      <c r="S91" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="T91" s="11" t="n"/>
       <c r="U91" s="11" t="n"/>
       <c r="V91" s="11" t="n"/>
       <c r="W91" s="11" t="n"/>
       <c r="X91" s="11" t="n"/>
-      <c r="Y91" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="13" t="inlineStr">
-        <is>
-          <t>世界半導体市場は26年2月に大幅成長、日本のみ9カ月連続マイナスに：全体は前年比61.8％増</t>
-        </is>
-      </c>
-      <c r="B92" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C92" s="15" t="n"/>
-      <c r="D92" s="15" t="n"/>
-      <c r="E92" s="15" t="n"/>
-      <c r="F92" s="15" t="n"/>
-      <c r="G92" s="15" t="n"/>
-      <c r="H92" s="15" t="n"/>
-      <c r="I92" s="15" t="n"/>
-      <c r="J92" s="15" t="n"/>
-      <c r="K92" s="15" t="n"/>
-      <c r="L92" s="15" t="n"/>
-      <c r="M92" s="15" t="n"/>
-      <c r="N92" s="15" t="n"/>
-      <c r="O92" s="15" t="n"/>
-      <c r="P92" s="15" t="n"/>
-      <c r="Q92" s="15" t="n"/>
-      <c r="R92" s="15" t="n"/>
-      <c r="S92" s="15" t="n"/>
-      <c r="T92" s="15" t="n"/>
-      <c r="U92" s="15" t="n"/>
-      <c r="V92" s="15" t="n"/>
-      <c r="W92" s="15" t="n"/>
-      <c r="X92" s="15" t="n"/>
-      <c r="Y92" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="9" t="inlineStr">
-        <is>
-          <t>半導体市場の成長| 2035 年の規模、トレンド、洞察</t>
-        </is>
-      </c>
-      <c r="B93" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C93" s="11" t="n"/>
-      <c r="D93" s="11" t="n"/>
-      <c r="E93" s="11" t="n"/>
-      <c r="F93" s="11" t="n"/>
-      <c r="G93" s="11" t="n"/>
-      <c r="H93" s="11" t="n"/>
-      <c r="I93" s="11" t="n"/>
-      <c r="J93" s="11" t="n"/>
-      <c r="K93" s="11" t="n"/>
-      <c r="L93" s="11" t="n"/>
-      <c r="M93" s="11" t="n"/>
-      <c r="N93" s="11" t="n"/>
-      <c r="O93" s="11" t="n"/>
-      <c r="P93" s="11" t="n"/>
-      <c r="Q93" s="11" t="n"/>
-      <c r="R93" s="11" t="n"/>
-      <c r="S93" s="11" t="n"/>
-      <c r="T93" s="11" t="n"/>
-      <c r="U93" s="11" t="n"/>
-      <c r="V93" s="11" t="n"/>
-      <c r="W93" s="11" t="n"/>
-      <c r="X93" s="11" t="n"/>
-      <c r="Y93" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="13" t="inlineStr">
-        <is>
-          <t>内閣府と経産省、第2回AI・半導体ワーキンググループ開催 バーティカルAIなどへの投資を議論</t>
-        </is>
-      </c>
-      <c r="B94" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C94" s="15" t="n"/>
-      <c r="D94" s="15" t="n"/>
-      <c r="E94" s="15" t="n"/>
-      <c r="F94" s="15" t="n"/>
-      <c r="G94" s="15" t="n"/>
-      <c r="H94" s="15" t="n"/>
-      <c r="I94" s="15" t="n"/>
-      <c r="J94" s="15" t="n"/>
-      <c r="K94" s="15" t="n"/>
-      <c r="L94" s="15" t="n"/>
-      <c r="M94" s="15" t="n"/>
-      <c r="N94" s="15" t="n"/>
-      <c r="O94" s="15" t="n"/>
-      <c r="P94" s="15" t="n"/>
-      <c r="Q94" s="15" t="n"/>
-      <c r="R94" s="15" t="n"/>
-      <c r="S94" s="15" t="n"/>
-      <c r="T94" s="15" t="n"/>
-      <c r="U94" s="15" t="n"/>
-      <c r="V94" s="15" t="n"/>
-      <c r="W94" s="15" t="n"/>
-      <c r="X94" s="15" t="n"/>
-      <c r="Y94" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="9" t="inlineStr">
-        <is>
-          <t>AIを軸に日本にチャンス到来、データセンター投資、半導体材料が活発に</t>
-        </is>
-      </c>
-      <c r="B95" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C95" s="11" t="n"/>
-      <c r="D95" s="11" t="n"/>
-      <c r="E95" s="11" t="n"/>
-      <c r="F95" s="11" t="n"/>
-      <c r="G95" s="11" t="n"/>
-      <c r="H95" s="11" t="n"/>
-      <c r="I95" s="11" t="n"/>
-      <c r="J95" s="11" t="n"/>
-      <c r="K95" s="11" t="n"/>
-      <c r="L95" s="11" t="n"/>
-      <c r="M95" s="11" t="n"/>
-      <c r="N95" s="11" t="n"/>
-      <c r="O95" s="11" t="n"/>
-      <c r="P95" s="11" t="n"/>
-      <c r="Q95" s="11" t="n"/>
-      <c r="R95" s="11" t="n"/>
-      <c r="S95" s="11" t="n"/>
-      <c r="T95" s="11" t="n"/>
-      <c r="U95" s="11" t="n"/>
-      <c r="V95" s="11" t="n"/>
-      <c r="W95" s="11" t="n"/>
-      <c r="X95" s="11" t="n"/>
-      <c r="Y95" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="13" t="inlineStr">
-        <is>
-          <t>一般電子部品の日本市場（～2031年）、市場規模（能動部品、受動部品、電気機械部品）・分析レポートを発表</t>
-        </is>
-      </c>
-      <c r="B96" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C96" s="15" t="n"/>
-      <c r="D96" s="15" t="n"/>
-      <c r="E96" s="15" t="n"/>
-      <c r="F96" s="15" t="n"/>
-      <c r="G96" s="15" t="n"/>
-      <c r="H96" s="15" t="n"/>
-      <c r="I96" s="15" t="n"/>
-      <c r="J96" s="15" t="n"/>
-      <c r="K96" s="15" t="n"/>
-      <c r="L96" s="15" t="n"/>
-      <c r="M96" s="15" t="n"/>
-      <c r="N96" s="15" t="n"/>
-      <c r="O96" s="15" t="n"/>
-      <c r="P96" s="15" t="n"/>
-      <c r="Q96" s="15" t="n"/>
-      <c r="R96" s="15" t="n"/>
-      <c r="S96" s="15" t="n"/>
-      <c r="T96" s="15" t="n"/>
-      <c r="U96" s="15" t="n"/>
-      <c r="V96" s="15" t="n"/>
-      <c r="W96" s="15" t="n"/>
-      <c r="X96" s="15" t="n"/>
-      <c r="Y96" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="9" t="inlineStr">
-        <is>
-          <t>堀場製作所は実は半導体の「ニッチトップ」企業！世界シェア6割を握る機器とは？創業家3代目が絶好調の受注環境を激白、問われるアクティビストへの対応力</t>
-        </is>
-      </c>
-      <c r="B97" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C97" s="11" t="n"/>
-      <c r="D97" s="11" t="n"/>
-      <c r="E97" s="11" t="n"/>
-      <c r="F97" s="11" t="n"/>
-      <c r="G97" s="11" t="n"/>
-      <c r="H97" s="11" t="n"/>
-      <c r="I97" s="11" t="n"/>
-      <c r="J97" s="11" t="n"/>
-      <c r="K97" s="11" t="n"/>
-      <c r="L97" s="11" t="n"/>
-      <c r="M97" s="11" t="n"/>
-      <c r="N97" s="11" t="n"/>
-      <c r="O97" s="11" t="n"/>
-      <c r="P97" s="11" t="n"/>
-      <c r="Q97" s="11" t="n"/>
-      <c r="R97" s="11" t="n"/>
-      <c r="S97" s="11" t="n"/>
-      <c r="T97" s="11" t="n"/>
-      <c r="U97" s="11" t="n"/>
-      <c r="V97" s="11" t="n"/>
-      <c r="W97" s="11" t="n"/>
-      <c r="X97" s="11" t="n"/>
-      <c r="Y97" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="13" t="inlineStr">
-        <is>
-          <t>オプテックスグループ[6914]：シーシーエスが自動車・半導体検査ソリューションの展示会を東海地方のお客様向けに開催 2026年4月6日(適時開示) ：日経会社情報DIGITAL</t>
-        </is>
-      </c>
-      <c r="B98" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C98" s="15" t="n"/>
-      <c r="D98" s="15" t="n"/>
-      <c r="E98" s="15" t="n"/>
-      <c r="F98" s="15" t="n"/>
-      <c r="G98" s="15" t="n"/>
-      <c r="H98" s="15" t="n"/>
-      <c r="I98" s="15" t="n"/>
-      <c r="J98" s="15" t="n"/>
-      <c r="K98" s="15" t="n"/>
-      <c r="L98" s="15" t="n"/>
-      <c r="M98" s="15" t="n"/>
-      <c r="N98" s="15" t="n"/>
-      <c r="O98" s="15" t="n"/>
-      <c r="P98" s="15" t="n"/>
-      <c r="Q98" s="15" t="n"/>
-      <c r="R98" s="15" t="n"/>
-      <c r="S98" s="15" t="n"/>
-      <c r="T98" s="15" t="n"/>
-      <c r="U98" s="15" t="n"/>
-      <c r="V98" s="15" t="n"/>
-      <c r="W98" s="15" t="n"/>
-      <c r="X98" s="15" t="n"/>
-      <c r="Y98" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="9" t="inlineStr">
-        <is>
-          <t>半導体アセンブリおよびテストサービス市場規模[2028]</t>
-        </is>
-      </c>
-      <c r="B99" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C99" s="11" t="n"/>
-      <c r="D99" s="11" t="n"/>
-      <c r="E99" s="11" t="n"/>
-      <c r="F99" s="11" t="n"/>
-      <c r="G99" s="11" t="n"/>
-      <c r="H99" s="11" t="n"/>
-      <c r="I99" s="11" t="n"/>
-      <c r="J99" s="11" t="n"/>
-      <c r="K99" s="11" t="n"/>
-      <c r="L99" s="11" t="n"/>
-      <c r="M99" s="11" t="n"/>
-      <c r="N99" s="11" t="n"/>
-      <c r="O99" s="11" t="n"/>
-      <c r="P99" s="11" t="n"/>
-      <c r="Q99" s="11" t="n"/>
-      <c r="R99" s="11" t="n"/>
-      <c r="S99" s="11" t="n"/>
-      <c r="T99" s="11" t="n"/>
-      <c r="U99" s="11" t="n"/>
-      <c r="V99" s="11" t="n"/>
-      <c r="W99" s="11" t="n"/>
-      <c r="X99" s="11" t="n"/>
-      <c r="Y99" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="13" t="inlineStr">
-        <is>
-          <t>シーシーエスが自動車・半導体検査ソリューションの展示会を 東海地方のお客様向けに開催</t>
-        </is>
-      </c>
-      <c r="B100" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-06</t>
-        </is>
-      </c>
-      <c r="C100" s="15" t="n"/>
-      <c r="D100" s="15" t="n"/>
-      <c r="E100" s="15" t="n"/>
-      <c r="F100" s="15" t="n"/>
-      <c r="G100" s="15" t="n"/>
-      <c r="H100" s="15" t="n"/>
-      <c r="I100" s="15" t="n"/>
-      <c r="J100" s="15" t="n"/>
-      <c r="K100" s="15" t="n"/>
-      <c r="L100" s="15" t="n"/>
-      <c r="M100" s="15" t="n"/>
-      <c r="N100" s="15" t="n"/>
-      <c r="O100" s="15" t="n"/>
-      <c r="P100" s="15" t="n"/>
-      <c r="Q100" s="15" t="n"/>
-      <c r="R100" s="15" t="n"/>
-      <c r="S100" s="15" t="n"/>
-      <c r="T100" s="15" t="n"/>
-      <c r="U100" s="15" t="n"/>
-      <c r="V100" s="15" t="n"/>
-      <c r="W100" s="15" t="n"/>
-      <c r="X100" s="15" t="n"/>
-      <c r="Y100" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="9" t="inlineStr">
-        <is>
-          <t>米議員グループ、対中半導体装置輸出の規制強化法案を公表</t>
-        </is>
-      </c>
-      <c r="B101" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-05</t>
-        </is>
-      </c>
-      <c r="C101" s="11" t="n"/>
-      <c r="D101" s="11" t="n"/>
-      <c r="E101" s="11" t="n"/>
-      <c r="F101" s="11" t="n"/>
-      <c r="G101" s="11" t="n"/>
-      <c r="H101" s="11" t="n"/>
-      <c r="I101" s="11" t="n"/>
-      <c r="J101" s="11" t="n"/>
-      <c r="K101" s="11" t="n"/>
-      <c r="L101" s="11" t="n"/>
-      <c r="M101" s="11" t="n"/>
-      <c r="N101" s="11" t="n"/>
-      <c r="O101" s="11" t="n"/>
-      <c r="P101" s="11" t="n"/>
-      <c r="Q101" s="11" t="n"/>
-      <c r="R101" s="11" t="n"/>
-      <c r="S101" s="11" t="n"/>
-      <c r="T101" s="11" t="n"/>
-      <c r="U101" s="11" t="n"/>
-      <c r="V101" s="11" t="n"/>
-      <c r="W101" s="11" t="n"/>
-      <c r="X101" s="11" t="n"/>
-      <c r="Y101" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="13" t="inlineStr">
-        <is>
-          <t>マイクロソフト、日本の AI 主導型成長に 1 兆 6000 億円を投資。AI インフラ、国家安全保障、人材育成を通じたさらなる国力強化を支援</t>
-        </is>
-      </c>
-      <c r="B102" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-03</t>
-        </is>
-      </c>
-      <c r="C102" s="15" t="n"/>
-      <c r="D102" s="15" t="n"/>
-      <c r="E102" s="15" t="n"/>
-      <c r="F102" s="15" t="n"/>
-      <c r="G102" s="15" t="n"/>
-      <c r="H102" s="15" t="n"/>
-      <c r="I102" s="15" t="n"/>
-      <c r="J102" s="15" t="n"/>
-      <c r="K102" s="15" t="n"/>
-      <c r="L102" s="15" t="n"/>
-      <c r="M102" s="15" t="n"/>
-      <c r="N102" s="15" t="n"/>
-      <c r="O102" s="15" t="n"/>
-      <c r="P102" s="15" t="n"/>
-      <c r="Q102" s="15" t="n"/>
-      <c r="R102" s="15" t="n"/>
-      <c r="S102" s="15" t="n"/>
-      <c r="T102" s="15" t="n"/>
-      <c r="U102" s="15" t="n"/>
-      <c r="V102" s="15" t="n"/>
-      <c r="W102" s="15" t="n"/>
-      <c r="X102" s="15" t="n"/>
-      <c r="Y102" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="9" t="inlineStr">
-        <is>
-          <t>2026年、27年とも300mm工場への設備投資は2桁成長～SEMI予測</t>
-        </is>
-      </c>
-      <c r="B103" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-03</t>
-        </is>
-      </c>
-      <c r="C103" s="11" t="n"/>
-      <c r="D103" s="11" t="n"/>
-      <c r="E103" s="11" t="n"/>
-      <c r="F103" s="11" t="n"/>
-      <c r="G103" s="11" t="n"/>
-      <c r="H103" s="11" t="n"/>
-      <c r="I103" s="11" t="n"/>
-      <c r="J103" s="11" t="n"/>
-      <c r="K103" s="11" t="n"/>
-      <c r="L103" s="11" t="n"/>
-      <c r="M103" s="11" t="n"/>
-      <c r="N103" s="11" t="n"/>
-      <c r="O103" s="11" t="n"/>
-      <c r="P103" s="11" t="n"/>
-      <c r="Q103" s="11" t="n"/>
-      <c r="R103" s="11" t="n"/>
-      <c r="S103" s="11" t="n"/>
-      <c r="T103" s="11" t="n"/>
-      <c r="U103" s="11" t="n"/>
-      <c r="V103" s="11" t="n"/>
-      <c r="W103" s="11" t="n"/>
-      <c r="X103" s="11" t="n"/>
-      <c r="Y103" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="13" t="inlineStr">
-        <is>
-          <t>中国ＡＩ半導体市場、国内勢がシェア4割強 エヌビディア優位性縮小</t>
-        </is>
-      </c>
-      <c r="B104" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="C104" s="15" t="n"/>
-      <c r="D104" s="15" t="n"/>
-      <c r="E104" s="15" t="n"/>
-      <c r="F104" s="15" t="n"/>
-      <c r="G104" s="15" t="n"/>
-      <c r="H104" s="15" t="n"/>
-      <c r="I104" s="15" t="n"/>
-      <c r="J104" s="15" t="n"/>
-      <c r="K104" s="15" t="n"/>
-      <c r="L104" s="15" t="n"/>
-      <c r="M104" s="15" t="n"/>
-      <c r="N104" s="15" t="n"/>
-      <c r="O104" s="15" t="n"/>
-      <c r="P104" s="15" t="n"/>
-      <c r="Q104" s="15" t="n"/>
-      <c r="R104" s="15" t="n"/>
-      <c r="S104" s="15" t="n"/>
-      <c r="T104" s="15" t="n"/>
-      <c r="U104" s="15" t="n"/>
-      <c r="V104" s="15" t="n"/>
-      <c r="W104" s="15" t="n"/>
-      <c r="X104" s="15" t="n"/>
-      <c r="Y104" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="9" t="inlineStr">
-        <is>
-          <t>競争激しい半導体市場へ…日本ガイシが4月から『NGK』に 社名変更の背景に“祖業からのシフトチェンジ”（東海テレビ）</t>
-        </is>
-      </c>
-      <c r="B105" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="C105" s="11" t="n"/>
-      <c r="D105" s="11" t="n"/>
-      <c r="E105" s="11" t="n"/>
-      <c r="F105" s="11" t="n"/>
-      <c r="G105" s="11" t="n"/>
-      <c r="H105" s="11" t="n"/>
-      <c r="I105" s="11" t="n"/>
-      <c r="J105" s="11" t="n"/>
-      <c r="K105" s="11" t="n"/>
-      <c r="L105" s="11" t="n"/>
-      <c r="M105" s="11" t="n"/>
-      <c r="N105" s="11" t="n"/>
-      <c r="O105" s="11" t="n"/>
-      <c r="P105" s="11" t="n"/>
-      <c r="Q105" s="11" t="n"/>
-      <c r="R105" s="11" t="n"/>
-      <c r="S105" s="11" t="n"/>
-      <c r="T105" s="11" t="n"/>
-      <c r="U105" s="11" t="n"/>
-      <c r="V105" s="11" t="n"/>
-      <c r="W105" s="11" t="n"/>
-      <c r="X105" s="11" t="n"/>
-      <c r="Y105" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="13" t="inlineStr">
-        <is>
-          <t>世界の供給網に「ヘリウムショック」 MRI検査からAI半導体まで波及</t>
-        </is>
-      </c>
-      <c r="B106" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="C106" s="15" t="n"/>
-      <c r="D106" s="15" t="n"/>
-      <c r="E106" s="15" t="n"/>
-      <c r="F106" s="15" t="n"/>
-      <c r="G106" s="15" t="n"/>
-      <c r="H106" s="15" t="n"/>
-      <c r="I106" s="15" t="n"/>
-      <c r="J106" s="15" t="n"/>
-      <c r="K106" s="15" t="n"/>
-      <c r="L106" s="15" t="n"/>
-      <c r="M106" s="15" t="n"/>
-      <c r="N106" s="15" t="n"/>
-      <c r="O106" s="15" t="n"/>
-      <c r="P106" s="15" t="n"/>
-      <c r="Q106" s="15" t="n"/>
-      <c r="R106" s="15" t="n"/>
-      <c r="S106" s="15" t="n"/>
-      <c r="T106" s="15" t="n"/>
-      <c r="U106" s="15" t="n"/>
-      <c r="V106" s="15" t="n"/>
-      <c r="W106" s="15" t="n"/>
-      <c r="X106" s="15" t="n"/>
-      <c r="Y106" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="9" t="inlineStr">
-        <is>
-          <t>アドテスト、ユーロ円建てＣＢ1000億円 半導体検査装置の生産能力増強</t>
-        </is>
-      </c>
-      <c r="B107" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="C107" s="11" t="n"/>
-      <c r="D107" s="11" t="n"/>
-      <c r="E107" s="11" t="n"/>
-      <c r="F107" s="11" t="n"/>
-      <c r="G107" s="11" t="n"/>
-      <c r="H107" s="11" t="n"/>
-      <c r="I107" s="11" t="n"/>
-      <c r="J107" s="11" t="n"/>
-      <c r="K107" s="11" t="n"/>
-      <c r="L107" s="11" t="n"/>
-      <c r="M107" s="11" t="n"/>
-      <c r="N107" s="11" t="n"/>
-      <c r="O107" s="11" t="n"/>
-      <c r="P107" s="11" t="n"/>
-      <c r="Q107" s="11" t="n"/>
-      <c r="R107" s="11" t="n"/>
-      <c r="S107" s="11" t="n"/>
-      <c r="T107" s="11" t="n"/>
-      <c r="U107" s="11" t="n"/>
-      <c r="V107" s="11" t="n"/>
-      <c r="W107" s="11" t="n"/>
-      <c r="X107" s="11" t="n"/>
-      <c r="Y107" s="12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="13" t="inlineStr">
-        <is>
-          <t>半導体製造は日本企業の技術が必須 業界マップで投資先探し</t>
-        </is>
-      </c>
-      <c r="B108" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="C108" s="15" t="n"/>
-      <c r="D108" s="15" t="n"/>
-      <c r="E108" s="15" t="n"/>
-      <c r="F108" s="15" t="n"/>
-      <c r="G108" s="15" t="n"/>
-      <c r="H108" s="15" t="n"/>
-      <c r="I108" s="15" t="n"/>
-      <c r="J108" s="15" t="n"/>
-      <c r="K108" s="15" t="n"/>
-      <c r="L108" s="15" t="n"/>
-      <c r="M108" s="15" t="n"/>
-      <c r="N108" s="15" t="n"/>
-      <c r="O108" s="15" t="n"/>
-      <c r="P108" s="15" t="n"/>
-      <c r="Q108" s="15" t="n"/>
-      <c r="R108" s="15" t="n"/>
-      <c r="S108" s="15" t="n"/>
-      <c r="T108" s="15" t="n"/>
-      <c r="U108" s="15" t="n"/>
-      <c r="V108" s="15" t="n"/>
-      <c r="W108" s="15" t="n"/>
-      <c r="X108" s="15" t="n"/>
-      <c r="Y108" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="9" t="inlineStr">
-        <is>
-          <t>半導体ウェハ検査技術のPhoto electron Soul、約9億円の資金調達を完了</t>
-        </is>
-      </c>
-      <c r="B109" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="C109" s="11" t="n"/>
-      <c r="D109" s="11" t="n"/>
-      <c r="E109" s="11" t="n"/>
-      <c r="F109" s="11" t="n"/>
-      <c r="G109" s="11" t="n"/>
-      <c r="H109" s="11" t="n"/>
-      <c r="I109" s="11" t="n"/>
-      <c r="J109" s="11" t="n"/>
-      <c r="K109" s="11" t="n"/>
-      <c r="L109" s="11" t="n"/>
-      <c r="M109" s="11" t="n"/>
-      <c r="N109" s="11" t="n"/>
-      <c r="O109" s="11" t="n"/>
-      <c r="P109" s="11" t="n"/>
-      <c r="Q109" s="11" t="n"/>
-      <c r="R109" s="11" t="n"/>
-      <c r="S109" s="11" t="n"/>
-      <c r="T109" s="11" t="n"/>
-      <c r="U109" s="11" t="n"/>
-      <c r="V109" s="11" t="n"/>
-      <c r="W109" s="11" t="n"/>
-      <c r="X109" s="11" t="n"/>
-      <c r="Y109" s="12" t="n">
-        <v>1</v>
-      </c>
+      <c r="Y91" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -4866,24 +4420,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A89" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A90" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A91" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A92" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A93" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A94" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A95" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A96" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A97" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A98" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A100" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A101" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A102" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A103" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A104" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A105" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A106" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A107" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A108" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A109" r:id="rId107"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>